<commit_message>
fix: lazy-load google drive auth to prevent startup crash
</commit_message>
<xml_diff>
--- a/My Job/LAPORAN KEGIATAN.xlsx
+++ b/My Job/LAPORAN KEGIATAN.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9302"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27932"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Smart Volunteers PMI Kota Cilegon\My Job\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7BB4C3F9-D2E2-4B47-BC0F-E189A1EDDFC8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="30" windowWidth="20115" windowHeight="7485"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="19440" windowHeight="14880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -12,6 +18,11 @@
     <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="144525"/>
+  <extLst>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -432,12 +443,12 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="4">
-    <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
-    <numFmt numFmtId="41" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;_);_(@_)"/>
-    <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="166" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="164" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
+    <numFmt numFmtId="165" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;_);_(@_)"/>
+    <numFmt numFmtId="166" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="167" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
   <fonts count="15" x14ac:knownFonts="1">
     <font>
@@ -680,9 +691,9 @@
   <cellStyleXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="81">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -786,14 +797,14 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1"/>
+    <xf numFmtId="167" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1"/>
     <xf numFmtId="3" fontId="4" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="3" fontId="4" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="4" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="4" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -802,7 +813,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="4" fillId="3" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="4" fillId="3" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -835,13 +846,13 @@
     <xf numFmtId="3" fontId="4" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="6" fillId="3" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="6" fillId="3" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="4" fillId="3" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="4" fillId="3" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="10" fillId="4" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="10" fillId="4" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="4" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -850,13 +861,13 @@
     <xf numFmtId="0" fontId="11" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="11" fillId="4" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="11" fillId="4" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="1" fontId="4" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="4" fillId="3" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="4" fillId="3" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -902,6 +913,9 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="4" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -909,18 +923,15 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="5">
-    <cellStyle name="Comma [0] 2" xfId="3"/>
-    <cellStyle name="Comma 2" xfId="2"/>
-    <cellStyle name="Currency [0] 2" xfId="4"/>
+    <cellStyle name="Comma [0] 2" xfId="3" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
+    <cellStyle name="Comma 2" xfId="2" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
+    <cellStyle name="Currency [0] 2" xfId="4" xr:uid="{00000000-0005-0000-0000-000002000000}"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 2" xfId="1"/>
+    <cellStyle name="Normal 2" xfId="1" xr:uid="{00000000-0005-0000-0000-000004000000}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -928,14 +939,17 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
     </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
   </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -973,7 +987,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -1045,7 +1059,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1218,17 +1232,20 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:P113"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
+    <col min="2" max="2" width="16.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.42578125" customWidth="1"/>
     <col min="4" max="4" width="18.7109375" customWidth="1"/>
     <col min="5" max="6" width="5" customWidth="1"/>
     <col min="7" max="7" width="9.85546875" customWidth="1"/>
     <col min="8" max="8" width="5.7109375" customWidth="1"/>
     <col min="9" max="9" width="5" customWidth="1"/>
-    <col min="10" max="11" width="5.7109375" customWidth="1"/>
-    <col min="12" max="12" width="5.28515625" customWidth="1"/>
+    <col min="10" max="10" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="10" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8.7109375" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="10" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="29" customWidth="1"/>
     <col min="15" max="15" width="13" customWidth="1"/>
@@ -1337,28 +1354,28 @@
       <c r="B6" s="80" t="s">
         <v>4</v>
       </c>
-      <c r="C6" s="79" t="s">
+      <c r="C6" s="77" t="s">
         <v>5</v>
       </c>
-      <c r="D6" s="79" t="s">
+      <c r="D6" s="77" t="s">
         <v>6</v>
       </c>
-      <c r="E6" s="79" t="s">
+      <c r="E6" s="77" t="s">
         <v>7</v>
       </c>
-      <c r="F6" s="79"/>
-      <c r="G6" s="79"/>
-      <c r="H6" s="79"/>
-      <c r="I6" s="79"/>
-      <c r="J6" s="79" t="s">
+      <c r="F6" s="77"/>
+      <c r="G6" s="77"/>
+      <c r="H6" s="77"/>
+      <c r="I6" s="77"/>
+      <c r="J6" s="77" t="s">
         <v>8</v>
       </c>
-      <c r="K6" s="79"/>
-      <c r="L6" s="79" t="s">
+      <c r="K6" s="77"/>
+      <c r="L6" s="77" t="s">
         <v>9</v>
       </c>
-      <c r="M6" s="79"/>
-      <c r="N6" s="79" t="s">
+      <c r="M6" s="77"/>
+      <c r="N6" s="77" t="s">
         <v>10</v>
       </c>
       <c r="O6" s="80" t="s">
@@ -1366,11 +1383,11 @@
       </c>
       <c r="P6" s="1"/>
     </row>
-    <row r="7" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7" s="80"/>
       <c r="B7" s="80"/>
-      <c r="C7" s="79"/>
-      <c r="D7" s="79"/>
+      <c r="C7" s="77"/>
+      <c r="D7" s="77"/>
       <c r="E7" s="45" t="s">
         <v>12</v>
       </c>
@@ -1398,7 +1415,7 @@
       <c r="M7" s="44" t="s">
         <v>20</v>
       </c>
-      <c r="N7" s="79"/>
+      <c r="N7" s="77"/>
       <c r="O7" s="80"/>
       <c r="P7" s="1"/>
     </row>
@@ -1422,7 +1439,7 @@
       <c r="O8" s="47"/>
       <c r="P8" s="37"/>
     </row>
-    <row r="9" spans="1:16" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:16" ht="165" x14ac:dyDescent="0.25">
       <c r="A9" s="41">
         <v>1</v>
       </c>
@@ -1468,7 +1485,7 @@
       </c>
       <c r="P9" s="37"/>
     </row>
-    <row r="10" spans="1:16" ht="270" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:16" ht="75" x14ac:dyDescent="0.25">
       <c r="A10" s="41">
         <v>2</v>
       </c>
@@ -1514,7 +1531,7 @@
       </c>
       <c r="P10" s="37"/>
     </row>
-    <row r="11" spans="1:16" ht="255" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:16" ht="90" x14ac:dyDescent="0.25">
       <c r="A11" s="41">
         <v>3</v>
       </c>
@@ -1556,7 +1573,7 @@
       </c>
       <c r="P11" s="37"/>
     </row>
-    <row r="12" spans="1:16" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:16" ht="120" x14ac:dyDescent="0.25">
       <c r="A12" s="41"/>
       <c r="B12" s="8">
         <v>46042</v>
@@ -1590,7 +1607,7 @@
       </c>
       <c r="P12" s="37"/>
     </row>
-    <row r="13" spans="1:16" ht="105" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:16" ht="45" x14ac:dyDescent="0.25">
       <c r="A13" s="41"/>
       <c r="B13" s="8">
         <v>46053</v>
@@ -1623,12 +1640,12 @@
       <c r="P13" s="37"/>
     </row>
     <row r="14" spans="1:16" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A14" s="77" t="s">
+      <c r="A14" s="78" t="s">
         <v>39</v>
       </c>
-      <c r="B14" s="78"/>
-      <c r="C14" s="78"/>
-      <c r="D14" s="78"/>
+      <c r="B14" s="79"/>
+      <c r="C14" s="79"/>
+      <c r="D14" s="79"/>
       <c r="E14" s="58">
         <v>48</v>
       </c>
@@ -1805,7 +1822,7 @@
       </c>
       <c r="O21" s="31"/>
     </row>
-    <row r="22" spans="1:15" ht="300" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:15" ht="75" x14ac:dyDescent="0.3">
       <c r="A22" s="31"/>
       <c r="B22" s="31" t="s">
         <v>45</v>
@@ -1865,7 +1882,7 @@
       <c r="N23" s="47"/>
       <c r="O23" s="47"/>
     </row>
-    <row r="24" spans="1:15" ht="120" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:15" ht="105" x14ac:dyDescent="0.3">
       <c r="A24" s="10"/>
       <c r="B24" s="34">
         <v>46142</v>
@@ -1965,7 +1982,7 @@
       </c>
       <c r="O27" s="66"/>
     </row>
-    <row r="28" spans="1:15" ht="240" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:15" ht="75" x14ac:dyDescent="0.25">
       <c r="A28" s="27"/>
       <c r="B28" s="65" t="s">
         <v>56</v>
@@ -2095,7 +2112,7 @@
       <c r="N33" s="47"/>
       <c r="O33" s="47"/>
     </row>
-    <row r="34" spans="1:15" ht="75" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:15" ht="45" x14ac:dyDescent="0.25">
       <c r="A34" s="10"/>
       <c r="B34" s="30" t="s">
         <v>66</v>
@@ -2130,7 +2147,7 @@
       </c>
       <c r="O34" s="39"/>
     </row>
-    <row r="35" spans="1:15" ht="75" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:15" ht="45" x14ac:dyDescent="0.25">
       <c r="A35" s="10"/>
       <c r="B35" s="30" t="s">
         <v>70</v>
@@ -2596,37 +2613,37 @@
       <c r="B60" s="80" t="s">
         <v>4</v>
       </c>
-      <c r="C60" s="79" t="s">
+      <c r="C60" s="77" t="s">
         <v>5</v>
       </c>
-      <c r="D60" s="79" t="s">
+      <c r="D60" s="77" t="s">
         <v>6</v>
       </c>
-      <c r="E60" s="79" t="s">
+      <c r="E60" s="77" t="s">
         <v>7</v>
       </c>
-      <c r="F60" s="79"/>
-      <c r="G60" s="79"/>
-      <c r="H60" s="79"/>
-      <c r="I60" s="79"/>
-      <c r="J60" s="79" t="s">
+      <c r="F60" s="77"/>
+      <c r="G60" s="77"/>
+      <c r="H60" s="77"/>
+      <c r="I60" s="77"/>
+      <c r="J60" s="77" t="s">
         <v>8</v>
       </c>
-      <c r="K60" s="79"/>
+      <c r="K60" s="77"/>
       <c r="L60" s="44"/>
       <c r="M60" s="44"/>
-      <c r="N60" s="79" t="s">
+      <c r="N60" s="77" t="s">
         <v>10</v>
       </c>
       <c r="O60" s="80" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="61" spans="1:15" ht="30" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A61" s="80"/>
       <c r="B61" s="80"/>
-      <c r="C61" s="79"/>
-      <c r="D61" s="79"/>
+      <c r="C61" s="77"/>
+      <c r="D61" s="77"/>
       <c r="E61" s="45" t="s">
         <v>12</v>
       </c>
@@ -2650,7 +2667,7 @@
       </c>
       <c r="L61" s="44"/>
       <c r="M61" s="44"/>
-      <c r="N61" s="79"/>
+      <c r="N61" s="77"/>
       <c r="O61" s="80"/>
     </row>
     <row r="62" spans="1:15" x14ac:dyDescent="0.25">
@@ -2672,7 +2689,7 @@
       <c r="N62" s="47"/>
       <c r="O62" s="47"/>
     </row>
-    <row r="63" spans="1:15" ht="195" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:15" ht="75" x14ac:dyDescent="0.25">
       <c r="A63" s="41"/>
       <c r="B63" s="8">
         <v>46046</v>
@@ -3022,7 +3039,7 @@
       <c r="N78" s="49"/>
       <c r="O78" s="49"/>
     </row>
-    <row r="79" spans="1:15" ht="120" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:15" ht="115.5" x14ac:dyDescent="0.3">
       <c r="A79" s="10"/>
       <c r="B79" s="30" t="s">
         <v>52</v>
@@ -3099,7 +3116,7 @@
       <c r="N81" s="47"/>
       <c r="O81" s="47"/>
     </row>
-    <row r="82" spans="1:15" ht="135" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:15" ht="90" x14ac:dyDescent="0.35">
       <c r="A82" s="10"/>
       <c r="B82" s="30" t="s">
         <v>97</v>
@@ -3126,7 +3143,7 @@
       </c>
       <c r="O82" s="39"/>
     </row>
-    <row r="83" spans="1:15" ht="105" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:15" ht="45" x14ac:dyDescent="0.25">
       <c r="A83" s="10"/>
       <c r="B83" s="30" t="s">
         <v>101</v>
@@ -3793,6 +3810,8 @@
     </row>
   </sheetData>
   <mergeCells count="18">
+    <mergeCell ref="C60:C61"/>
+    <mergeCell ref="D60:D61"/>
     <mergeCell ref="J60:K60"/>
     <mergeCell ref="E60:I60"/>
     <mergeCell ref="A14:D14"/>
@@ -3809,15 +3828,13 @@
     <mergeCell ref="J6:K6"/>
     <mergeCell ref="A60:A61"/>
     <mergeCell ref="B60:B61"/>
-    <mergeCell ref="C60:C61"/>
-    <mergeCell ref="D60:D61"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
@@ -3826,7 +3843,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>

</xml_diff>